<commit_message>
feat: implement pricing plan and localization
</commit_message>
<xml_diff>
--- a/public/data/technicians.xlsx
+++ b/public/data/technicians.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,9 +410,6 @@
         <v>group</v>
       </c>
       <c r="D1" t="str">
-        <v>base_price</v>
-      </c>
-      <c r="E1" t="str">
         <v>active</v>
       </c>
     </row>
@@ -426,10 +423,7 @@
       <c r="C2" t="str">
         <v>Group A</v>
       </c>
-      <c r="D2">
-        <v>2400</v>
-      </c>
-      <c r="E2" t="b">
+      <c r="D2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -443,10 +437,7 @@
       <c r="C3" t="str">
         <v>Group A</v>
       </c>
-      <c r="D3">
-        <v>2400</v>
-      </c>
-      <c r="E3" t="b">
+      <c r="D3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -460,10 +451,7 @@
       <c r="C4" t="str">
         <v>Group A</v>
       </c>
-      <c r="D4">
-        <v>2400</v>
-      </c>
-      <c r="E4" t="b">
+      <c r="D4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -477,10 +465,7 @@
       <c r="C5" t="str">
         <v>Group A</v>
       </c>
-      <c r="D5">
-        <v>2400</v>
-      </c>
-      <c r="E5" t="b">
+      <c r="D5" t="b">
         <v>1</v>
       </c>
     </row>
@@ -494,10 +479,7 @@
       <c r="C6" t="str">
         <v>Group A</v>
       </c>
-      <c r="D6">
-        <v>2000</v>
-      </c>
-      <c r="E6" t="b">
+      <c r="D6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -511,10 +493,7 @@
       <c r="C7" t="str">
         <v>Group B</v>
       </c>
-      <c r="D7">
-        <v>2000</v>
-      </c>
-      <c r="E7" t="b">
+      <c r="D7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -528,10 +507,7 @@
       <c r="C8" t="str">
         <v>Group B</v>
       </c>
-      <c r="D8">
-        <v>2800</v>
-      </c>
-      <c r="E8" t="b">
+      <c r="D8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -545,10 +521,7 @@
       <c r="C9" t="str">
         <v>Group B</v>
       </c>
-      <c r="D9">
-        <v>2000</v>
-      </c>
-      <c r="E9" t="b">
+      <c r="D9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -562,16 +535,13 @@
       <c r="C10" t="str">
         <v>Group C</v>
       </c>
-      <c r="D10">
-        <v>1500</v>
-      </c>
-      <c r="E10" t="b">
+      <c r="D10" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>